<commit_message>
data: refresh grade summary
</commit_message>
<xml_diff>
--- a/grades_summary.xlsx
+++ b/grades_summary.xlsx
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>3317.6</v>
@@ -690,19 +690,19 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>4023.8</v>
+        <v>5338.3</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>2837.6</v>
+        <v>4753</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>229945</v>
+        <v>222962</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>140046</v>
+        <v>244693</v>
       </c>
     </row>
     <row r="14">
@@ -3855,24 +3855,22 @@
         </is>
       </c>
       <c r="C124" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D124" s="3" t="n">
         <v>6</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>483.2</v>
+        <v>478.3</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>119.8</v>
+        <v>268.5</v>
       </c>
       <c r="G124" s="3" t="n">
-        <v>26653</v>
-      </c>
-      <c r="H124" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>18410</v>
+      </c>
+      <c r="H124" s="3" t="n">
+        <v>18773</v>
       </c>
     </row>
     <row r="125">
@@ -4709,24 +4707,24 @@
         </is>
       </c>
       <c r="C154" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D154" s="3" t="n">
         <v>5</v>
       </c>
       <c r="E154" s="3" t="n">
-        <v>588.9</v>
+        <v>1492.4</v>
       </c>
       <c r="F154" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="G154" s="3" t="n">
-        <v>21868</v>
-      </c>
-      <c r="H154" s="3" t="inlineStr">
+        <v>1698.3</v>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>79936</v>
       </c>
     </row>
     <row r="155">
@@ -5853,20 +5851,16 @@
         <v>17</v>
       </c>
       <c r="E194" s="3" t="n">
-        <v>0</v>
+        <v>416</v>
       </c>
       <c r="F194" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G194" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H194" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>99.5</v>
+      </c>
+      <c r="G194" s="3" t="n">
+        <v>23128</v>
+      </c>
+      <c r="H194" s="3" t="n">
+        <v>5938</v>
       </c>
     </row>
     <row r="195">
@@ -6105,7 +6099,7 @@
         </is>
       </c>
       <c r="C203" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D203" s="3" t="n">
         <v>17</v>

</xml_diff>

<commit_message>
data: fix glm q18 grade
</commit_message>
<xml_diff>
--- a/grades_summary.xlsx
+++ b/grades_summary.xlsx
@@ -620,89 +620,89 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
         <v>146</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1762.5</v>
+        <v>5338.3</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>264.2</v>
+        <v>4694.3</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>173527</v>
+        <v>222962</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>37049</v>
+        <v>243948</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
         <v>146</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1085.7</v>
+        <v>1762.5</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>913.3</v>
+        <v>264.2</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>145855</v>
+        <v>173527</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>126064</v>
+        <v>37049</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
         <v>146</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>3317.6</v>
+        <v>1085.7</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2723.9</v>
+        <v>913.3</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>139635</v>
+        <v>145855</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>131401</v>
+        <v>126064</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>5338.3</v>
+        <v>3317.6</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4753</v>
+        <v>2723.9</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>222962</v>
+        <v>139635</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>244693</v>
+        <v>131401</v>
       </c>
     </row>
     <row r="14">
@@ -919,7 +919,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -929,16 +929,16 @@
         <v>5</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>316</v>
+        <v>364</v>
       </c>
     </row>
     <row r="22">
@@ -949,7 +949,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -959,16 +959,16 @@
         <v>5</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>6.7</v>
+        <v>1.8</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>5.3</v>
+        <v>2.1</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>308</v>
+        <v>316</v>
       </c>
     </row>
     <row r="23">
@@ -979,7 +979,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -989,16 +989,16 @@
         <v>5</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>3.8</v>
+        <v>6.7</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>15.8</v>
+        <v>5.3</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>334</v>
+        <v>286</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>362</v>
+        <v>308</v>
       </c>
     </row>
     <row r="24">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -1019,16 +1019,16 @@
         <v>5</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>4.1</v>
+        <v>15.8</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="25">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
@@ -1213,16 +1213,16 @@
         <v>5</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>2.2</v>
+        <v>14.3</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>2.3</v>
+        <v>8</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>360</v>
+        <v>538</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>360</v>
+        <v>714</v>
       </c>
     </row>
     <row r="32">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
@@ -1243,16 +1243,16 @@
         <v>5</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>9.9</v>
+        <v>2.2</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>6.8</v>
+        <v>2.3</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>596</v>
+        <v>360</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>548</v>
+        <v>360</v>
       </c>
     </row>
     <row r="33">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -1273,16 +1273,16 @@
         <v>5</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>6.7</v>
+        <v>9.9</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>8</v>
+        <v>6.8</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>491</v>
+        <v>596</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>457</v>
+        <v>548</v>
       </c>
     </row>
     <row r="34">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
@@ -1303,16 +1303,16 @@
         <v>5</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>14.3</v>
+        <v>6.7</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>8</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>538</v>
+        <v>491</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>714</v>
+        <v>457</v>
       </c>
     </row>
     <row r="35">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -1497,16 +1497,16 @@
         <v>5</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>4.2</v>
+        <v>10.5</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>4</v>
+        <v>16.9</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>700</v>
+        <v>971</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>662</v>
+        <v>913</v>
       </c>
     </row>
     <row r="42">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -1527,16 +1527,16 @@
         <v>5</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>9</v>
+        <v>4.2</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>10.2</v>
+        <v>4</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>858</v>
+        <v>700</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>787</v>
+        <v>662</v>
       </c>
     </row>
     <row r="43">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -1557,16 +1557,16 @@
         <v>5</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>3.2</v>
+        <v>10.2</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1082</v>
+        <v>787</v>
       </c>
     </row>
     <row r="44">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -1587,16 +1587,16 @@
         <v>5</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>10.5</v>
+        <v>10.8</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>16.9</v>
+        <v>3.2</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>971</v>
+        <v>856</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>913</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="45">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -1781,16 +1781,16 @@
         <v>5</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>2.7</v>
+        <v>7.5</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>422</v>
+        <v>562</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>369</v>
+        <v>659</v>
       </c>
     </row>
     <row r="52">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -1811,16 +1811,16 @@
         <v>5</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>6.7</v>
+        <v>3</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>14.2</v>
+        <v>2.7</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>670</v>
+        <v>422</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>594</v>
+        <v>369</v>
       </c>
     </row>
     <row r="53">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -1841,16 +1841,16 @@
         <v>5</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>6.7</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>14.2</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>522</v>
+        <v>670</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>624</v>
+        <v>594</v>
       </c>
     </row>
     <row r="54">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -1871,16 +1871,16 @@
         <v>5</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>562</v>
+        <v>522</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>659</v>
+        <v>624</v>
       </c>
     </row>
     <row r="55">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -2065,16 +2065,16 @@
         <v>5</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>5.1</v>
+        <v>15.2</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>5.9</v>
+        <v>15.6</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>763</v>
+        <v>1065</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>860</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="62">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -2095,16 +2095,16 @@
         <v>5</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>5.1</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>10.3</v>
+        <v>5.9</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>1236</v>
+        <v>763</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>1030</v>
+        <v>860</v>
       </c>
     </row>
     <row r="63">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -2125,16 +2125,16 @@
         <v>5</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>15.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>50.2</v>
+        <v>10.3</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>795</v>
+        <v>1236</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>2092</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="64">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
@@ -2155,16 +2155,16 @@
         <v>5</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>15.2</v>
+        <v>15.9</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>15.6</v>
+        <v>50.2</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>1065</v>
+        <v>795</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>1171</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="65">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -2349,16 +2349,16 @@
         <v>5</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>15.6</v>
+        <v>40.7</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>1.7</v>
+        <v>75.3</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>1508</v>
+        <v>2773</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="72">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -2379,16 +2379,16 @@
         <v>5</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>15.9</v>
+        <v>15.6</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>17.7</v>
+        <v>1.7</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>2034</v>
+        <v>1508</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>1965</v>
+        <v>405</v>
       </c>
     </row>
     <row r="73">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
@@ -2409,18 +2409,16 @@
         <v>5</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.6</v>
+        <v>15.9</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>158.8</v>
-      </c>
-      <c r="G73" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>17.7</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>2034</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>3836</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="74">
@@ -2431,7 +2429,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C74" s="3" t="n">
@@ -2441,16 +2439,18 @@
         <v>5</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>40.7</v>
+        <v>0.6</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>75.3</v>
-      </c>
-      <c r="G74" s="3" t="n">
-        <v>2773</v>
+        <v>158.8</v>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H74" s="3" t="n">
-        <v>1655</v>
+        <v>3836</v>
       </c>
     </row>
     <row r="75">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C81" s="3" t="n">
@@ -2635,16 +2635,16 @@
         <v>5</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>29.9</v>
+        <v>205.5</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>17.6</v>
+        <v>24.7</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>3358</v>
+        <v>13822</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>2165</v>
+        <v>3254</v>
       </c>
     </row>
     <row r="82">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C82" s="3" t="n">
@@ -2665,16 +2665,16 @@
         <v>5</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>32.4</v>
+        <v>29.9</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>11.2</v>
+        <v>17.6</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>4548</v>
+        <v>3358</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>2426</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="83">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C83" s="3" t="n">
@@ -2695,16 +2695,16 @@
         <v>5</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>26</v>
+        <v>32.4</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>45.3</v>
+        <v>11.2</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>5517</v>
+        <v>4548</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>3336</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="84">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C84" s="3" t="n">
@@ -2725,16 +2725,16 @@
         <v>5</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>205.5</v>
+        <v>26</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>24.7</v>
+        <v>45.3</v>
       </c>
       <c r="G84" s="3" t="n">
-        <v>13822</v>
+        <v>5517</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>3254</v>
+        <v>3336</v>
       </c>
     </row>
     <row r="85">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C91" s="3" t="n">
@@ -2919,16 +2919,16 @@
         <v>5</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>6.1</v>
+        <v>26.8</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>6.7</v>
+        <v>16.3</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>850</v>
+        <v>1072</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>806</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="92">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C92" s="3" t="n">
@@ -2949,16 +2949,16 @@
         <v>5</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>16.2</v>
+        <v>6.1</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>7.4</v>
+        <v>6.7</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>2050</v>
+        <v>850</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>1247</v>
+        <v>806</v>
       </c>
     </row>
     <row r="93">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C93" s="3" t="n">
@@ -2979,16 +2979,16 @@
         <v>5</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>39</v>
+        <v>16.2</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>31.4</v>
+        <v>7.4</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>1268</v>
+        <v>2050</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>1373</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="94">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C94" s="3" t="n">
@@ -3009,16 +3009,16 @@
         <v>5</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>26.8</v>
+        <v>39</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>16.3</v>
+        <v>31.4</v>
       </c>
       <c r="G94" s="3" t="n">
-        <v>1072</v>
+        <v>1268</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>1228</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="95">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
@@ -3203,16 +3203,16 @@
         <v>6</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>7.5</v>
+        <v>16.8</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>4.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>927</v>
+        <v>1723</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>554</v>
+        <v>578</v>
       </c>
     </row>
     <row r="102">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C102" s="3" t="n">
@@ -3233,16 +3233,16 @@
         <v>6</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>10.6</v>
+        <v>7.5</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>4.7</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>975</v>
+        <v>927</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>1053</v>
+        <v>554</v>
       </c>
     </row>
     <row r="103">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C103" s="3" t="n">
@@ -3263,16 +3263,16 @@
         <v>6</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>36.6</v>
+        <v>10.6</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>12.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>1274</v>
+        <v>975</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>573</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="104">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C104" s="3" t="n">
@@ -3293,16 +3293,16 @@
         <v>6</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>16.8</v>
+        <v>36.6</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>12.1</v>
       </c>
       <c r="G104" s="3" t="n">
-        <v>1723</v>
+        <v>1274</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>578</v>
+        <v>573</v>
       </c>
     </row>
     <row r="105">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C111" s="3" t="n">
@@ -3487,16 +3487,16 @@
         <v>6</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>176.6</v>
+        <v>519.4</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>39.1</v>
+        <v>189.5</v>
       </c>
       <c r="G111" s="3" t="n">
-        <v>14518</v>
+        <v>16277</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>3873</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="112">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C112" s="3" t="n">
@@ -3517,16 +3517,16 @@
         <v>6</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>49.9</v>
+        <v>176.6</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>37</v>
+        <v>39.1</v>
       </c>
       <c r="G112" s="3" t="n">
-        <v>6708</v>
+        <v>14518</v>
       </c>
       <c r="H112" s="3" t="n">
-        <v>4710</v>
+        <v>3873</v>
       </c>
     </row>
     <row r="113">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C113" s="3" t="n">
@@ -3547,16 +3547,16 @@
         <v>6</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>392.3</v>
+        <v>49.9</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>398.7</v>
+        <v>37</v>
       </c>
       <c r="G113" s="3" t="n">
-        <v>11350</v>
+        <v>6708</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>15371</v>
+        <v>4710</v>
       </c>
     </row>
     <row r="114">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C114" s="3" t="n">
@@ -3577,16 +3577,16 @@
         <v>6</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>519.4</v>
+        <v>392.3</v>
       </c>
       <c r="F114" s="3" t="n">
-        <v>189.5</v>
+        <v>398.7</v>
       </c>
       <c r="G114" s="3" t="n">
-        <v>16277</v>
+        <v>11350</v>
       </c>
       <c r="H114" s="3" t="n">
-        <v>3854</v>
+        <v>15371</v>
       </c>
     </row>
     <row r="115">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C121" s="3" t="n">
@@ -3771,16 +3771,16 @@
         <v>6</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>223.3</v>
+        <v>478.3</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>39.8</v>
+        <v>268.5</v>
       </c>
       <c r="G121" s="3" t="n">
-        <v>22236</v>
+        <v>18410</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>4754</v>
+        <v>18773</v>
       </c>
     </row>
     <row r="122">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C122" s="3" t="n">
@@ -3801,16 +3801,16 @@
         <v>6</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>136.1</v>
+        <v>223.3</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>106.2</v>
+        <v>39.8</v>
       </c>
       <c r="G122" s="3" t="n">
-        <v>16351</v>
+        <v>22236</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>16382</v>
+        <v>4754</v>
       </c>
     </row>
     <row r="123">
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C123" s="3" t="n">
@@ -3831,16 +3831,16 @@
         <v>6</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>485.2</v>
+        <v>136.1</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>369.9</v>
+        <v>106.2</v>
       </c>
       <c r="G123" s="3" t="n">
-        <v>21109</v>
+        <v>16351</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>17164</v>
+        <v>16382</v>
       </c>
     </row>
     <row r="124">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C124" s="3" t="n">
@@ -3861,16 +3861,16 @@
         <v>6</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>478.3</v>
+        <v>485.2</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>268.5</v>
+        <v>369.9</v>
       </c>
       <c r="G124" s="3" t="n">
-        <v>18410</v>
+        <v>21109</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>18773</v>
+        <v>17164</v>
       </c>
     </row>
     <row r="125">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C131" s="3" t="n">
@@ -4055,16 +4055,16 @@
         <v>5</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>5.9</v>
+        <v>18.4</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>4</v>
+        <v>8.4</v>
       </c>
       <c r="G131" s="3" t="n">
-        <v>707</v>
+        <v>1180</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>541</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="132">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C132" s="3" t="n">
@@ -4085,16 +4085,16 @@
         <v>5</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>8.1</v>
+        <v>5.9</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>6.6</v>
+        <v>4</v>
       </c>
       <c r="G132" s="3" t="n">
-        <v>894</v>
+        <v>707</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>562</v>
+        <v>541</v>
       </c>
     </row>
     <row r="133">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C133" s="3" t="n">
@@ -4115,16 +4115,16 @@
         <v>5</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>97.2</v>
+        <v>8.1</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>15.5</v>
+        <v>6.6</v>
       </c>
       <c r="G133" s="3" t="n">
-        <v>2162</v>
+        <v>894</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>789</v>
+        <v>562</v>
       </c>
     </row>
     <row r="134">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C134" s="3" t="n">
@@ -4145,16 +4145,16 @@
         <v>5</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>18.4</v>
+        <v>97.2</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>8.4</v>
+        <v>15.5</v>
       </c>
       <c r="G134" s="3" t="n">
-        <v>1180</v>
+        <v>2162</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>1144</v>
+        <v>789</v>
       </c>
     </row>
     <row r="135">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C141" s="3" t="n">
@@ -4339,16 +4339,16 @@
         <v>5</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>76.7</v>
+        <v>276.6</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>34.5</v>
+        <v>151.4</v>
       </c>
       <c r="G141" s="3" t="n">
-        <v>7598</v>
+        <v>15030</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>3523</v>
+        <v>8329</v>
       </c>
     </row>
     <row r="142">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C142" s="3" t="n">
@@ -4369,16 +4369,16 @@
         <v>5</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>51.3</v>
+        <v>76.7</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>47.4</v>
+        <v>34.5</v>
       </c>
       <c r="G142" s="3" t="n">
-        <v>6643</v>
+        <v>7598</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>5905</v>
+        <v>3523</v>
       </c>
     </row>
     <row r="143">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C143" s="3" t="n">
@@ -4399,16 +4399,16 @@
         <v>5</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>107.2</v>
+        <v>51.3</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>62.2</v>
+        <v>47.4</v>
       </c>
       <c r="G143" s="3" t="n">
-        <v>6821</v>
+        <v>6643</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>4665</v>
+        <v>5905</v>
       </c>
     </row>
     <row r="144">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C144" s="3" t="n">
@@ -4429,16 +4429,16 @@
         <v>5</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>276.6</v>
+        <v>107.2</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>151.4</v>
+        <v>62.2</v>
       </c>
       <c r="G144" s="3" t="n">
-        <v>15030</v>
+        <v>6821</v>
       </c>
       <c r="H144" s="3" t="n">
-        <v>8329</v>
+        <v>4665</v>
       </c>
     </row>
     <row r="145">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C151" s="3" t="n">
@@ -4623,16 +4623,18 @@
         <v>5</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>161.4</v>
+        <v>1492.4</v>
       </c>
       <c r="F151" s="3" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="G151" s="3" t="n">
-        <v>15111</v>
+        <v>1698.3</v>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="H151" s="3" t="n">
-        <v>4907</v>
+        <v>79936</v>
       </c>
     </row>
     <row r="152">
@@ -4643,7 +4645,7 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C152" s="3" t="n">
@@ -4653,16 +4655,16 @@
         <v>5</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>113.7</v>
+        <v>161.4</v>
       </c>
       <c r="F152" s="3" t="n">
-        <v>167.5</v>
+        <v>46.1</v>
       </c>
       <c r="G152" s="3" t="n">
-        <v>15519</v>
+        <v>15111</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>11931</v>
+        <v>4907</v>
       </c>
     </row>
     <row r="153">
@@ -4673,7 +4675,7 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C153" s="3" t="n">
@@ -4683,16 +4685,16 @@
         <v>5</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>394.8</v>
+        <v>113.7</v>
       </c>
       <c r="F153" s="3" t="n">
-        <v>140</v>
+        <v>167.5</v>
       </c>
       <c r="G153" s="3" t="n">
-        <v>22505</v>
+        <v>15519</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>6934</v>
+        <v>11931</v>
       </c>
     </row>
     <row r="154">
@@ -4703,7 +4705,7 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C154" s="3" t="n">
@@ -4713,18 +4715,16 @@
         <v>5</v>
       </c>
       <c r="E154" s="3" t="n">
-        <v>1492.4</v>
+        <v>394.8</v>
       </c>
       <c r="F154" s="3" t="n">
-        <v>1698.3</v>
-      </c>
-      <c r="G154" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>140</v>
+      </c>
+      <c r="G154" s="3" t="n">
+        <v>22505</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>79936</v>
+        <v>6934</v>
       </c>
     </row>
     <row r="155">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C161" s="3" t="n">
@@ -4909,16 +4909,16 @@
         <v>13</v>
       </c>
       <c r="E161" s="3" t="n">
-        <v>28</v>
+        <v>487</v>
       </c>
       <c r="F161" s="3" t="n">
-        <v>4.7</v>
+        <v>19.5</v>
       </c>
       <c r="G161" s="3" t="n">
-        <v>3444</v>
+        <v>10146</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>1982</v>
+        <v>4412</v>
       </c>
     </row>
     <row r="162">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C162" s="3" t="n">
@@ -4939,16 +4939,16 @@
         <v>13</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>54.9</v>
+        <v>28</v>
       </c>
       <c r="F162" s="3" t="n">
-        <v>20.1</v>
+        <v>4.7</v>
       </c>
       <c r="G162" s="3" t="n">
-        <v>8663</v>
+        <v>3444</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>4530</v>
+        <v>1982</v>
       </c>
     </row>
     <row r="163">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C163" s="3" t="n">
@@ -4969,16 +4969,16 @@
         <v>13</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>248.7</v>
+        <v>54.9</v>
       </c>
       <c r="F163" s="3" t="n">
-        <v>109.2</v>
+        <v>20.1</v>
       </c>
       <c r="G163" s="3" t="n">
-        <v>10894</v>
+        <v>8663</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>4779</v>
+        <v>4530</v>
       </c>
     </row>
     <row r="164">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C164" s="3" t="n">
@@ -4999,16 +4999,16 @@
         <v>13</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>487</v>
+        <v>248.7</v>
       </c>
       <c r="F164" s="3" t="n">
-        <v>19.5</v>
+        <v>109.2</v>
       </c>
       <c r="G164" s="3" t="n">
-        <v>10146</v>
+        <v>10894</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>4412</v>
+        <v>4779</v>
       </c>
     </row>
     <row r="165">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C171" s="3" t="n">
@@ -5193,16 +5193,16 @@
         <v>15</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>37.1</v>
+        <v>109.6</v>
       </c>
       <c r="F171" s="3" t="n">
-        <v>15</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="G171" s="3" t="n">
-        <v>4059</v>
+        <v>6854</v>
       </c>
       <c r="H171" s="3" t="n">
-        <v>2493</v>
+        <v>6159</v>
       </c>
     </row>
     <row r="172">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C172" s="3" t="n">
@@ -5223,16 +5223,16 @@
         <v>15</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>118.4</v>
+        <v>37.1</v>
       </c>
       <c r="F172" s="3" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="G172" s="3" t="n">
-        <v>16111</v>
+        <v>4059</v>
       </c>
       <c r="H172" s="3" t="n">
-        <v>8307</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="173">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C173" s="3" t="n">
@@ -5253,16 +5253,16 @@
         <v>15</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>271.7</v>
+        <v>118.4</v>
       </c>
       <c r="F173" s="3" t="n">
-        <v>286.9</v>
+        <v>54</v>
       </c>
       <c r="G173" s="3" t="n">
-        <v>9644</v>
+        <v>16111</v>
       </c>
       <c r="H173" s="3" t="n">
-        <v>9986</v>
+        <v>8307</v>
       </c>
     </row>
     <row r="174">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C174" s="3" t="n">
@@ -5283,16 +5283,16 @@
         <v>15</v>
       </c>
       <c r="E174" s="3" t="n">
-        <v>109.6</v>
+        <v>271.7</v>
       </c>
       <c r="F174" s="3" t="n">
-        <v>64.40000000000001</v>
+        <v>286.9</v>
       </c>
       <c r="G174" s="3" t="n">
-        <v>6854</v>
+        <v>9644</v>
       </c>
       <c r="H174" s="3" t="n">
-        <v>6159</v>
+        <v>9986</v>
       </c>
     </row>
     <row r="175">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C181" s="3" t="n">
@@ -5477,16 +5477,16 @@
         <v>15</v>
       </c>
       <c r="E181" s="3" t="n">
-        <v>20.4</v>
+        <v>110.3</v>
       </c>
       <c r="F181" s="3" t="n">
-        <v>14.8</v>
+        <v>20.3</v>
       </c>
       <c r="G181" s="3" t="n">
-        <v>2367</v>
+        <v>7316</v>
       </c>
       <c r="H181" s="3" t="n">
-        <v>2584</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="182">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C182" s="3" t="n">
@@ -5507,16 +5507,16 @@
         <v>15</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>55.2</v>
+        <v>20.4</v>
       </c>
       <c r="F182" s="3" t="n">
-        <v>33.6</v>
+        <v>14.8</v>
       </c>
       <c r="G182" s="3" t="n">
-        <v>6668</v>
+        <v>2367</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>4885</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="183">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C183" s="3" t="n">
@@ -5537,16 +5537,16 @@
         <v>15</v>
       </c>
       <c r="E183" s="3" t="n">
-        <v>118.6</v>
+        <v>55.2</v>
       </c>
       <c r="F183" s="3" t="n">
-        <v>83.59999999999999</v>
+        <v>33.6</v>
       </c>
       <c r="G183" s="3" t="n">
-        <v>6904</v>
+        <v>6668</v>
       </c>
       <c r="H183" s="3" t="n">
-        <v>4233</v>
+        <v>4885</v>
       </c>
     </row>
     <row r="184">
@@ -5557,7 +5557,7 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C184" s="3" t="n">
@@ -5567,16 +5567,16 @@
         <v>15</v>
       </c>
       <c r="E184" s="3" t="n">
-        <v>110.3</v>
+        <v>118.6</v>
       </c>
       <c r="F184" s="3" t="n">
-        <v>20.3</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="G184" s="3" t="n">
-        <v>7316</v>
+        <v>6904</v>
       </c>
       <c r="H184" s="3" t="n">
-        <v>1940</v>
+        <v>4233</v>
       </c>
     </row>
     <row r="185">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C191" s="3" t="n">
@@ -5761,16 +5761,16 @@
         <v>17</v>
       </c>
       <c r="E191" s="3" t="n">
-        <v>130.5</v>
+        <v>416</v>
       </c>
       <c r="F191" s="3" t="n">
-        <v>8.9</v>
+        <v>40.7</v>
       </c>
       <c r="G191" s="3" t="n">
-        <v>12565</v>
+        <v>23128</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>2745</v>
+        <v>5193</v>
       </c>
     </row>
     <row r="192">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C192" s="3" t="n">
@@ -5791,16 +5791,16 @@
         <v>17</v>
       </c>
       <c r="E192" s="3" t="n">
-        <v>94.2</v>
+        <v>130.5</v>
       </c>
       <c r="F192" s="3" t="n">
-        <v>61.1</v>
+        <v>8.9</v>
       </c>
       <c r="G192" s="3" t="n">
-        <v>13383</v>
+        <v>12565</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>10991</v>
+        <v>2745</v>
       </c>
     </row>
     <row r="193">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C193" s="3" t="n">
@@ -5821,16 +5821,16 @@
         <v>17</v>
       </c>
       <c r="E193" s="3" t="n">
-        <v>451.8</v>
+        <v>94.2</v>
       </c>
       <c r="F193" s="3" t="n">
-        <v>238.3</v>
+        <v>61.1</v>
       </c>
       <c r="G193" s="3" t="n">
-        <v>16306</v>
+        <v>13383</v>
       </c>
       <c r="H193" s="3" t="n">
-        <v>9623</v>
+        <v>10991</v>
       </c>
     </row>
     <row r="194">
@@ -5841,26 +5841,26 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C194" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D194" s="3" t="n">
         <v>17</v>
       </c>
       <c r="E194" s="3" t="n">
-        <v>416</v>
+        <v>451.8</v>
       </c>
       <c r="F194" s="3" t="n">
-        <v>99.5</v>
+        <v>238.3</v>
       </c>
       <c r="G194" s="3" t="n">
-        <v>23128</v>
+        <v>16306</v>
       </c>
       <c r="H194" s="3" t="n">
-        <v>5938</v>
+        <v>9623</v>
       </c>
     </row>
     <row r="195">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C201" s="3" t="n">
@@ -6045,16 +6045,16 @@
         <v>17</v>
       </c>
       <c r="E201" s="3" t="n">
-        <v>827.4</v>
+        <v>1088.2</v>
       </c>
       <c r="F201" s="3" t="n">
-        <v>9.5</v>
+        <v>2056.1</v>
       </c>
       <c r="G201" s="3" t="n">
-        <v>81763</v>
+        <v>101816</v>
       </c>
       <c r="H201" s="3" t="n">
-        <v>3150</v>
+        <v>103672</v>
       </c>
     </row>
     <row r="202">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C202" s="3" t="n">
@@ -6075,16 +6075,16 @@
         <v>17</v>
       </c>
       <c r="E202" s="3" t="n">
-        <v>286.8</v>
+        <v>827.4</v>
       </c>
       <c r="F202" s="3" t="n">
-        <v>287.9</v>
+        <v>9.5</v>
       </c>
       <c r="G202" s="3" t="n">
-        <v>41662</v>
+        <v>81763</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>47903</v>
+        <v>3150</v>
       </c>
     </row>
     <row r="203">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C203" s="3" t="n">
@@ -6105,16 +6105,16 @@
         <v>17</v>
       </c>
       <c r="E203" s="3" t="n">
-        <v>602</v>
+        <v>286.8</v>
       </c>
       <c r="F203" s="3" t="n">
-        <v>685.2</v>
+        <v>287.9</v>
       </c>
       <c r="G203" s="3" t="n">
-        <v>20883</v>
+        <v>41662</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>44122</v>
+        <v>47903</v>
       </c>
     </row>
     <row r="204">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C204" s="3" t="n">
@@ -6135,16 +6135,16 @@
         <v>17</v>
       </c>
       <c r="E204" s="3" t="n">
-        <v>1088.2</v>
+        <v>602</v>
       </c>
       <c r="F204" s="3" t="n">
-        <v>2056.1</v>
+        <v>685.2</v>
       </c>
       <c r="G204" s="3" t="n">
-        <v>101816</v>
+        <v>20883</v>
       </c>
       <c r="H204" s="3" t="n">
-        <v>103672</v>
+        <v>44122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: fix glm national ii q18 grade
</commit_message>
<xml_diff>
--- a/grades_summary.xlsx
+++ b/grades_summary.xlsx
@@ -6213,177 +6213,177 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
         <v>150</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>568.1</v>
+        <v>1443.3</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>342.6</v>
+        <v>769.8</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>38446</v>
+        <v>98285</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>30162</v>
+        <v>68604</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
         <v>150</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>935.1</v>
+        <v>568.1</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>281.8</v>
+        <v>342.6</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>79812</v>
+        <v>38446</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>100018</v>
+        <v>30162</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
         <v>150</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1657.9</v>
+        <v>935.1</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>187.3</v>
+        <v>281.8</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>156124</v>
+        <v>79812</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>34310</v>
+        <v>100018</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
         <v>150</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2763.2</v>
+        <v>1657.9</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>599.8</v>
+        <v>187.3</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>167591</v>
+        <v>156124</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>55813</v>
+        <v>34310</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
         <v>150</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>591.5</v>
+        <v>2763.2</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>407.7</v>
+        <v>599.8</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>79685</v>
+        <v>167591</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>62148</v>
+        <v>55813</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
         <v>150</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2519.4</v>
+        <v>591.5</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1061.1</v>
+        <v>407.7</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>117778</v>
+        <v>79685</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>70914</v>
+        <v>62148</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>573.5</v>
+        <v>2519.4</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>200.4</v>
+        <v>1061.1</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>79929</v>
+        <v>117778</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>35537</v>
+        <v>70914</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1280.2</v>
+        <v>573.5</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>810.5</v>
+        <v>200.4</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>87584</v>
+        <v>79929</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>64658</v>
+        <v>35537</v>
       </c>
     </row>
     <row r="11">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -6482,16 +6482,16 @@
         <v>5</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4.2</v>
+        <v>3.2</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>4.6</v>
+        <v>3.6</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>250</v>
+        <v>315</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>274</v>
+        <v>346</v>
       </c>
     </row>
     <row r="17">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -6512,16 +6512,16 @@
         <v>5</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2.6</v>
+        <v>4.2</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -6542,16 +6542,16 @@
         <v>5</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>5.5</v>
+        <v>2.6</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>2.4</v>
+        <v>4.4</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>622</v>
+        <v>240</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>511</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19">
@@ -6562,7 +6562,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -6572,16 +6572,16 @@
         <v>5</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>10.8</v>
+        <v>5.5</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>8.4</v>
+        <v>2.4</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>690</v>
+        <v>622</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>670</v>
+        <v>511</v>
       </c>
     </row>
     <row r="20">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -6602,16 +6602,16 @@
         <v>5</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>4.8</v>
+        <v>10.8</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>4.9</v>
+        <v>8.4</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>409</v>
+        <v>690</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>363</v>
+        <v>670</v>
       </c>
     </row>
     <row r="21">
@@ -6622,7 +6622,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -6632,16 +6632,16 @@
         <v>5</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>9.1</v>
+        <v>4.8</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>3.1</v>
+        <v>4.9</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>461</v>
+        <v>409</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>858</v>
+        <v>363</v>
       </c>
     </row>
     <row r="22">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -6662,16 +6662,16 @@
         <v>5</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>2</v>
+        <v>9.1</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>1.7</v>
+        <v>3.1</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>324</v>
+        <v>461</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>320</v>
+        <v>858</v>
       </c>
     </row>
     <row r="23">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -6692,16 +6692,16 @@
         <v>5</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>3.6</v>
+        <v>1.7</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>346</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -6766,16 +6766,16 @@
         <v>5</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>3.6</v>
+        <v>9.9</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>313</v>
+        <v>680</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>338</v>
+        <v>523</v>
       </c>
     </row>
     <row r="27">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -6796,16 +6796,16 @@
         <v>5</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>6.3</v>
+        <v>3.6</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>2.2</v>
+        <v>5.5</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>604</v>
+        <v>313</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>640</v>
+        <v>338</v>
       </c>
     </row>
     <row r="28">
@@ -6816,7 +6816,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -6826,16 +6826,16 @@
         <v>5</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>5.6</v>
+        <v>6.3</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>595</v>
+        <v>604</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>389</v>
+        <v>640</v>
       </c>
     </row>
     <row r="29">
@@ -6846,7 +6846,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -6856,16 +6856,16 @@
         <v>5</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>8.1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>649</v>
+        <v>595</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>676</v>
+        <v>389</v>
       </c>
     </row>
     <row r="30">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
@@ -6886,16 +6886,16 @@
         <v>5</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>4.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>5.7</v>
+        <v>8.1</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>540</v>
+        <v>649</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>542</v>
+        <v>676</v>
       </c>
     </row>
     <row r="31">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
@@ -6916,16 +6916,16 @@
         <v>5</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>9.1</v>
+        <v>4.3</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>18.2</v>
+        <v>5.7</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>405</v>
+        <v>540</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>894</v>
+        <v>542</v>
       </c>
     </row>
     <row r="32">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
@@ -6946,16 +6946,16 @@
         <v>5</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>2.9</v>
+        <v>9.1</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>1.9</v>
+        <v>18.2</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>448</v>
+        <v>405</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>322</v>
+        <v>894</v>
       </c>
     </row>
     <row r="33">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -6976,16 +6976,16 @@
         <v>5</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>9.9</v>
+        <v>2.9</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>5.7</v>
+        <v>1.9</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>680</v>
+        <v>448</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>523</v>
+        <v>322</v>
       </c>
     </row>
     <row r="34">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
@@ -7050,16 +7050,16 @@
         <v>5</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>3</v>
+        <v>6.9</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>5.3</v>
+        <v>18</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>340</v>
+        <v>692</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>404</v>
+        <v>716</v>
       </c>
     </row>
     <row r="37">
@@ -7070,7 +7070,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -7080,16 +7080,16 @@
         <v>5</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>7.7</v>
+        <v>3</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>1.9</v>
+        <v>5.3</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>727</v>
+        <v>340</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>764</v>
+        <v>404</v>
       </c>
     </row>
     <row r="38">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
@@ -7110,16 +7110,16 @@
         <v>5</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>14.4</v>
+        <v>7.7</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>5.3</v>
+        <v>1.9</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>1199</v>
+        <v>727</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>578</v>
+        <v>764</v>
       </c>
     </row>
     <row r="39">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -7140,16 +7140,16 @@
         <v>5</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>19.2</v>
+        <v>14.4</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>5.8</v>
+        <v>5.3</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>1321</v>
+        <v>1199</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>978</v>
+        <v>578</v>
       </c>
     </row>
     <row r="40">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -7170,16 +7170,16 @@
         <v>5</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>6.7</v>
+        <v>19.2</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>8</v>
+        <v>5.8</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>934</v>
+        <v>1321</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>736</v>
+        <v>978</v>
       </c>
     </row>
     <row r="41">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -7200,16 +7200,16 @@
         <v>5</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>6.7</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>12.7</v>
+        <v>8</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>422</v>
+        <v>934</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>615</v>
+        <v>736</v>
       </c>
     </row>
     <row r="42">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -7230,16 +7230,16 @@
         <v>5</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>3.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>2.2</v>
+        <v>12.7</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>622</v>
+        <v>422</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>605</v>
+        <v>615</v>
       </c>
     </row>
     <row r="43">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -7260,16 +7260,16 @@
         <v>5</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>6.9</v>
+        <v>3.5</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>18</v>
+        <v>2.2</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>692</v>
+        <v>622</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>716</v>
+        <v>605</v>
       </c>
     </row>
     <row r="44">
@@ -7324,7 +7324,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -7334,16 +7334,16 @@
         <v>5</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>5</v>
+        <v>20.7</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>6</v>
+        <v>10.3</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>435</v>
+        <v>1336</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>466</v>
+        <v>860</v>
       </c>
     </row>
     <row r="47">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -7364,16 +7364,16 @@
         <v>5</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>7.1</v>
+        <v>5</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>723</v>
+        <v>435</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>760</v>
+        <v>466</v>
       </c>
     </row>
     <row r="48">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
@@ -7394,16 +7394,16 @@
         <v>5</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>15.8</v>
+        <v>7.1</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>1809</v>
+        <v>723</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>780</v>
+        <v>760</v>
       </c>
     </row>
     <row r="49">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -7424,16 +7424,16 @@
         <v>5</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>33.8</v>
+        <v>15.8</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>2098</v>
+        <v>1809</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>877</v>
+        <v>780</v>
       </c>
     </row>
     <row r="50">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -7454,16 +7454,16 @@
         <v>5</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>6.5</v>
+        <v>33.8</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>7.8</v>
+        <v>2.1</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>909</v>
+        <v>2098</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>895</v>
+        <v>877</v>
       </c>
     </row>
     <row r="51">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -7484,16 +7484,16 @@
         <v>5</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>15.1</v>
+        <v>6.5</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>4.5</v>
+        <v>7.8</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>764</v>
+        <v>909</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>833</v>
+        <v>895</v>
       </c>
     </row>
     <row r="52">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -7514,16 +7514,16 @@
         <v>5</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>3.4</v>
+        <v>15.1</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>2.8</v>
+        <v>4.5</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>643</v>
+        <v>764</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>602</v>
+        <v>833</v>
       </c>
     </row>
     <row r="53">
@@ -7534,7 +7534,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -7544,16 +7544,16 @@
         <v>5</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>20.7</v>
+        <v>3.4</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>10.3</v>
+        <v>2.8</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>1336</v>
+        <v>643</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>860</v>
+        <v>602</v>
       </c>
     </row>
     <row r="54">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -7618,16 +7618,16 @@
         <v>5</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>9</v>
+        <v>13.1</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>7.8</v>
+        <v>10.8</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>569</v>
+        <v>1598</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>574</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="57">
@@ -7638,7 +7638,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
@@ -7648,16 +7648,16 @@
         <v>5</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>25.5</v>
+        <v>9</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>2.4</v>
+        <v>7.8</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>2294</v>
+        <v>569</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>2331</v>
+        <v>574</v>
       </c>
     </row>
     <row r="58">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -7678,16 +7678,16 @@
         <v>5</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>66</v>
+        <v>25.5</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>6010</v>
+        <v>2294</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>956</v>
+        <v>2331</v>
       </c>
     </row>
     <row r="59">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
@@ -7708,16 +7708,16 @@
         <v>5</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>33.1</v>
+        <v>66</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>42.2</v>
+        <v>2.6</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>2039</v>
+        <v>6010</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>2826</v>
+        <v>956</v>
       </c>
     </row>
     <row r="60">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -7738,16 +7738,16 @@
         <v>5</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>15.2</v>
+        <v>33.1</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>8.5</v>
+        <v>42.2</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>1555</v>
+        <v>2039</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>1197</v>
+        <v>2826</v>
       </c>
     </row>
     <row r="61">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
@@ -7768,16 +7768,16 @@
         <v>5</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>45.2</v>
+        <v>15.2</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>29.2</v>
+        <v>8.5</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>2303</v>
+        <v>1555</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>1123</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="62">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
@@ -7798,16 +7798,16 @@
         <v>5</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>5.2</v>
+        <v>45.2</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>4.6</v>
+        <v>29.2</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>788</v>
+        <v>2303</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>792</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="63">
@@ -7818,7 +7818,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -7828,16 +7828,16 @@
         <v>5</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>13.1</v>
+        <v>5.2</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>10.8</v>
+        <v>4.6</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>1598</v>
+        <v>788</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>1673</v>
+        <v>792</v>
       </c>
     </row>
     <row r="64">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
@@ -7902,16 +7902,16 @@
         <v>5</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>6.7</v>
+        <v>16.5</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>6.9</v>
+        <v>9.9</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>530</v>
+        <v>2276</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>522</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="67">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
@@ -7932,16 +7932,16 @@
         <v>5</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>15.1</v>
+        <v>6.7</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>3</v>
+        <v>6.9</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>1020</v>
+        <v>530</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>1057</v>
+        <v>522</v>
       </c>
     </row>
     <row r="68">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
@@ -7962,16 +7962,16 @@
         <v>5</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>73.3</v>
+        <v>15.1</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>13.6</v>
+        <v>3</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>6070</v>
+        <v>1020</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>1695</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="69">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
@@ -7992,16 +7992,16 @@
         <v>5</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>121.4</v>
+        <v>73.3</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>55.1</v>
+        <v>13.6</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>6562</v>
+        <v>6070</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>3166</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="70">
@@ -8012,7 +8012,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -8022,16 +8022,16 @@
         <v>5</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>20.8</v>
+        <v>121.4</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>13.4</v>
+        <v>55.1</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>2656</v>
+        <v>6562</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>1619</v>
+        <v>3166</v>
       </c>
     </row>
     <row r="71">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
@@ -8052,16 +8052,16 @@
         <v>5</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>20.8</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>34.6</v>
+        <v>13.4</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>2377</v>
+        <v>2656</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>2346</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="72">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
@@ -8082,16 +8082,16 @@
         <v>5</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>14.5</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>13.7</v>
+        <v>34.6</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>1746</v>
+        <v>2377</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>1682</v>
+        <v>2346</v>
       </c>
     </row>
     <row r="73">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
@@ -8112,16 +8112,16 @@
         <v>5</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>16.5</v>
+        <v>14.5</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>9.9</v>
+        <v>13.7</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>2276</v>
+        <v>1746</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>1679</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="74">
@@ -8176,7 +8176,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C76" s="3" t="n">
@@ -8186,16 +8186,16 @@
         <v>5</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>6.4</v>
+        <v>21.3</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>8</v>
+        <v>3.1</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>548</v>
+        <v>1655</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>644</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="77">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C77" s="3" t="n">
@@ -8216,16 +8216,16 @@
         <v>5</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>19</v>
+        <v>6.4</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>1633</v>
+        <v>548</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>1670</v>
+        <v>644</v>
       </c>
     </row>
     <row r="78">
@@ -8236,7 +8236,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C78" s="3" t="n">
@@ -8246,16 +8246,16 @@
         <v>5</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>47.4</v>
+        <v>19</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>22.3</v>
+        <v>2</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>4384</v>
+        <v>1633</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>1831</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="79">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C79" s="3" t="n">
@@ -8276,16 +8276,16 @@
         <v>5</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>110.3</v>
+        <v>47.4</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>3</v>
+        <v>22.3</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>7730</v>
+        <v>4384</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>998</v>
+        <v>1831</v>
       </c>
     </row>
     <row r="80">
@@ -8296,7 +8296,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C80" s="3" t="n">
@@ -8306,16 +8306,16 @@
         <v>5</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>17</v>
+        <v>110.3</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>12.8</v>
+        <v>3</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>1628</v>
+        <v>7730</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>1488</v>
+        <v>998</v>
       </c>
     </row>
     <row r="81">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C81" s="3" t="n">
@@ -8336,16 +8336,16 @@
         <v>5</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>16.9</v>
+        <v>17</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>60.6</v>
+        <v>12.8</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>1005</v>
+        <v>1628</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>1845</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="82">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C82" s="3" t="n">
@@ -8366,16 +8366,16 @@
         <v>5</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>4.8</v>
+        <v>16.9</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>4.4</v>
+        <v>60.6</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>788</v>
+        <v>1005</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>765</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="83">
@@ -8386,7 +8386,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C83" s="3" t="n">
@@ -8396,16 +8396,16 @@
         <v>5</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>21.3</v>
+        <v>4.8</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>3.1</v>
+        <v>4.4</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>1655</v>
+        <v>788</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>1726</v>
+        <v>765</v>
       </c>
     </row>
     <row r="84">
@@ -8460,7 +8460,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C86" s="3" t="n">
@@ -8470,16 +8470,16 @@
         <v>5</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>18.1</v>
+        <v>19.1</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>26.1</v>
+        <v>71.7</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>1199</v>
+        <v>4273</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>1442</v>
+        <v>3806</v>
       </c>
     </row>
     <row r="87">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C87" s="3" t="n">
@@ -8500,16 +8500,16 @@
         <v>5</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>37.2</v>
+        <v>18.1</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>2.3</v>
+        <v>26.1</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>2726</v>
+        <v>1199</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>2763</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="88">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C88" s="3" t="n">
@@ -8530,16 +8530,16 @@
         <v>5</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>114.7</v>
+        <v>37.2</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>10135</v>
+        <v>2726</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>339</v>
+        <v>2763</v>
       </c>
     </row>
     <row r="89">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C89" s="3" t="n">
@@ -8560,16 +8560,16 @@
         <v>5</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>102</v>
+        <v>114.7</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>6463</v>
+        <v>10135</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>1226</v>
+        <v>339</v>
       </c>
     </row>
     <row r="90">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C90" s="3" t="n">
@@ -8590,16 +8590,16 @@
         <v>5</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>42.6</v>
+        <v>102</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>12</v>
+        <v>2.7</v>
       </c>
       <c r="G90" s="3" t="n">
-        <v>4246</v>
+        <v>6463</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>2235</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="91">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C91" s="3" t="n">
@@ -8620,16 +8620,16 @@
         <v>5</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>166.7</v>
+        <v>42.6</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>107.1</v>
+        <v>12</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>6708</v>
+        <v>4246</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>3957</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="92">
@@ -8640,7 +8640,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C92" s="3" t="n">
@@ -8650,16 +8650,16 @@
         <v>5</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>66.3</v>
+        <v>166.7</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>28.3</v>
+        <v>107.1</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>9687</v>
+        <v>6708</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>3716</v>
+        <v>3957</v>
       </c>
     </row>
     <row r="93">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C93" s="3" t="n">
@@ -8680,16 +8680,16 @@
         <v>5</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>19.1</v>
+        <v>66.3</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>71.7</v>
+        <v>28.3</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>4273</v>
+        <v>9687</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>3806</v>
+        <v>3716</v>
       </c>
     </row>
     <row r="94">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C96" s="3" t="n">
@@ -8754,16 +8754,16 @@
         <v>6</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>9.5</v>
+        <v>20.1</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="G96" s="3" t="n">
-        <v>704</v>
+        <v>2054</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>720</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="97">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C97" s="3" t="n">
@@ -8784,16 +8784,16 @@
         <v>6</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>21.2</v>
+        <v>9.5</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>2.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>1684</v>
+        <v>704</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>1721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="98">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C98" s="3" t="n">
@@ -8814,16 +8814,16 @@
         <v>6</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>72.7</v>
+        <v>21.2</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>6085</v>
+        <v>1684</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>918</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="99">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
@@ -8844,16 +8844,16 @@
         <v>6</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>72.2</v>
+        <v>72.7</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>5.1</v>
+        <v>1.6</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>4535</v>
+        <v>6085</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>1182</v>
+        <v>918</v>
       </c>
     </row>
     <row r="100">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C100" s="3" t="n">
@@ -8874,16 +8874,16 @@
         <v>6</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>22.4</v>
+        <v>72.2</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>19.9</v>
+        <v>5.1</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>2732</v>
+        <v>4535</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>2150</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="101">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
@@ -8904,16 +8904,16 @@
         <v>6</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>13.8</v>
+        <v>22.4</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>46.9</v>
+        <v>19.9</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>2586</v>
+        <v>2732</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>2319</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="102">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C102" s="3" t="n">
@@ -8934,16 +8934,16 @@
         <v>6</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>12.1</v>
+        <v>13.8</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>6.9</v>
+        <v>46.9</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>1448</v>
+        <v>2586</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>921</v>
+        <v>2319</v>
       </c>
     </row>
     <row r="103">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C103" s="3" t="n">
@@ -8964,16 +8964,16 @@
         <v>6</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>20.1</v>
+        <v>12.1</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>7.7</v>
+        <v>6.9</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>2054</v>
+        <v>1448</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>1905</v>
+        <v>921</v>
       </c>
     </row>
     <row r="104">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C106" s="3" t="n">
@@ -9038,16 +9038,16 @@
         <v>6</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>12.2</v>
+        <v>109.7</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>11.6</v>
+        <v>34.5</v>
       </c>
       <c r="G106" s="3" t="n">
-        <v>909</v>
+        <v>6503</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>975</v>
+        <v>2849</v>
       </c>
     </row>
     <row r="107">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C107" s="3" t="n">
@@ -9068,16 +9068,16 @@
         <v>6</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>27.5</v>
+        <v>12.2</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>9.6</v>
+        <v>11.6</v>
       </c>
       <c r="G107" s="3" t="n">
-        <v>2851</v>
+        <v>909</v>
       </c>
       <c r="H107" s="3" t="n">
-        <v>3430</v>
+        <v>975</v>
       </c>
     </row>
     <row r="108">
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C108" s="3" t="n">
@@ -9098,16 +9098,16 @@
         <v>6</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>103.2</v>
+        <v>27.5</v>
       </c>
       <c r="F108" s="3" t="n">
-        <v>19.7</v>
+        <v>9.6</v>
       </c>
       <c r="G108" s="3" t="n">
-        <v>8928</v>
+        <v>2851</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>2105</v>
+        <v>3430</v>
       </c>
     </row>
     <row r="109">
@@ -9118,7 +9118,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C109" s="3" t="n">
@@ -9128,16 +9128,16 @@
         <v>6</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>187</v>
+        <v>103.2</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>70</v>
+        <v>19.7</v>
       </c>
       <c r="G109" s="3" t="n">
-        <v>12297</v>
+        <v>8928</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>5884</v>
+        <v>2105</v>
       </c>
     </row>
     <row r="110">
@@ -9148,7 +9148,7 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C110" s="3" t="n">
@@ -9158,16 +9158,16 @@
         <v>6</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>23.8</v>
+        <v>187</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>33.8</v>
+        <v>70</v>
       </c>
       <c r="G110" s="3" t="n">
-        <v>3646</v>
+        <v>12297</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>4913</v>
+        <v>5884</v>
       </c>
     </row>
     <row r="111">
@@ -9178,7 +9178,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C111" s="3" t="n">
@@ -9188,16 +9188,16 @@
         <v>6</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>93.7</v>
+        <v>23.8</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>103.6</v>
+        <v>33.8</v>
       </c>
       <c r="G111" s="3" t="n">
-        <v>3548</v>
+        <v>3646</v>
       </c>
       <c r="H111" s="3" t="n">
-        <v>4335</v>
+        <v>4913</v>
       </c>
     </row>
     <row r="112">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C112" s="3" t="n">
@@ -9218,16 +9218,16 @@
         <v>6</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>15.8</v>
+        <v>93.7</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>12.8</v>
+        <v>103.6</v>
       </c>
       <c r="G112" s="3" t="n">
-        <v>2538</v>
+        <v>3548</v>
       </c>
       <c r="H112" s="3" t="n">
-        <v>2116</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="113">
@@ -9238,7 +9238,7 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C113" s="3" t="n">
@@ -9248,16 +9248,16 @@
         <v>6</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>109.7</v>
+        <v>15.8</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>34.5</v>
+        <v>12.8</v>
       </c>
       <c r="G113" s="3" t="n">
-        <v>6503</v>
+        <v>2538</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>2849</v>
+        <v>2116</v>
       </c>
     </row>
     <row r="114">
@@ -9312,7 +9312,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C116" s="3" t="n">
@@ -9322,16 +9322,16 @@
         <v>6</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>62.5</v>
+        <v>524.2</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>33.7</v>
+        <v>78.5</v>
       </c>
       <c r="G116" s="3" t="n">
-        <v>3418</v>
+        <v>23904</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>2144</v>
+        <v>9887</v>
       </c>
     </row>
     <row r="117">
@@ -9342,7 +9342,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C117" s="3" t="n">
@@ -9352,16 +9352,16 @@
         <v>6</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>196</v>
+        <v>62.5</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>105.9</v>
+        <v>33.7</v>
       </c>
       <c r="G117" s="3" t="n">
-        <v>16423</v>
+        <v>3418</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>24316</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="118">
@@ -9372,7 +9372,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C118" s="3" t="n">
@@ -9382,16 +9382,16 @@
         <v>6</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>216.7</v>
+        <v>196</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>19</v>
+        <v>105.9</v>
       </c>
       <c r="G118" s="3" t="n">
-        <v>20028</v>
+        <v>16423</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>1886</v>
+        <v>24316</v>
       </c>
     </row>
     <row r="119">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C119" s="3" t="n">
@@ -9412,16 +9412,16 @@
         <v>6</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>328.8</v>
+        <v>216.7</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>197.6</v>
+        <v>19</v>
       </c>
       <c r="G119" s="3" t="n">
-        <v>19450</v>
+        <v>20028</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>11378</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="120">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C120" s="3" t="n">
@@ -9442,16 +9442,16 @@
         <v>6</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>84.2</v>
+        <v>328.8</v>
       </c>
       <c r="F120" s="3" t="n">
-        <v>48.4</v>
+        <v>197.6</v>
       </c>
       <c r="G120" s="3" t="n">
-        <v>8288</v>
+        <v>19450</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>6857</v>
+        <v>11378</v>
       </c>
     </row>
     <row r="121">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C121" s="3" t="n">
@@ -9472,16 +9472,16 @@
         <v>6</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>204.8</v>
+        <v>84.2</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>166.7</v>
+        <v>48.4</v>
       </c>
       <c r="G121" s="3" t="n">
-        <v>12766</v>
+        <v>8288</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>9481</v>
+        <v>6857</v>
       </c>
     </row>
     <row r="122">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C122" s="3" t="n">
@@ -9502,16 +9502,16 @@
         <v>6</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>110.5</v>
+        <v>204.8</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>70.8</v>
+        <v>166.7</v>
       </c>
       <c r="G122" s="3" t="n">
-        <v>14685</v>
+        <v>12766</v>
       </c>
       <c r="H122" s="3" t="n">
-        <v>9016</v>
+        <v>9481</v>
       </c>
     </row>
     <row r="123">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C123" s="3" t="n">
@@ -9532,16 +9532,16 @@
         <v>6</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>524.2</v>
+        <v>110.5</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>78.5</v>
+        <v>70.8</v>
       </c>
       <c r="G123" s="3" t="n">
-        <v>23904</v>
+        <v>14685</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>9887</v>
+        <v>9016</v>
       </c>
     </row>
     <row r="124">
@@ -9596,7 +9596,7 @@
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C126" s="3" t="n">
@@ -9606,16 +9606,16 @@
         <v>5</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>3.5</v>
+        <v>16.2</v>
       </c>
       <c r="F126" s="3" t="n">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="G126" s="3" t="n">
-        <v>306</v>
+        <v>461</v>
       </c>
       <c r="H126" s="3" t="n">
-        <v>301</v>
+        <v>505</v>
       </c>
     </row>
     <row r="127">
@@ -9626,7 +9626,7 @@
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C127" s="3" t="n">
@@ -9636,16 +9636,16 @@
         <v>5</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>8.9</v>
+        <v>3.5</v>
       </c>
       <c r="F127" s="3" t="n">
-        <v>2.5</v>
+        <v>7.1</v>
       </c>
       <c r="G127" s="3" t="n">
-        <v>512</v>
+        <v>306</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>549</v>
+        <v>301</v>
       </c>
     </row>
     <row r="128">
@@ -9656,7 +9656,7 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C128" s="3" t="n">
@@ -9669,13 +9669,13 @@
         <v>8.9</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="G128" s="3" t="n">
-        <v>971</v>
+        <v>512</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>521</v>
+        <v>549</v>
       </c>
     </row>
     <row r="129">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C129" s="3" t="n">
@@ -9696,16 +9696,16 @@
         <v>5</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>19.8</v>
+        <v>8.9</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>4.1</v>
+        <v>1.3</v>
       </c>
       <c r="G129" s="3" t="n">
-        <v>1291</v>
+        <v>971</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>638</v>
+        <v>521</v>
       </c>
     </row>
     <row r="130">
@@ -9716,7 +9716,7 @@
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C130" s="3" t="n">
@@ -9726,16 +9726,16 @@
         <v>5</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>6.3</v>
+        <v>19.8</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>6.6</v>
+        <v>4.1</v>
       </c>
       <c r="G130" s="3" t="n">
-        <v>704</v>
+        <v>1291</v>
       </c>
       <c r="H130" s="3" t="n">
-        <v>552</v>
+        <v>638</v>
       </c>
     </row>
     <row r="131">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C131" s="3" t="n">
@@ -9756,16 +9756,16 @@
         <v>5</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>12.1</v>
+        <v>6.3</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>5.1</v>
+        <v>6.6</v>
       </c>
       <c r="G131" s="3" t="n">
-        <v>1110</v>
+        <v>704</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>625</v>
+        <v>552</v>
       </c>
     </row>
     <row r="132">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C132" s="3" t="n">
@@ -9786,16 +9786,16 @@
         <v>5</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>3.1</v>
+        <v>12.1</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>2.3</v>
+        <v>5.1</v>
       </c>
       <c r="G132" s="3" t="n">
-        <v>447</v>
+        <v>1110</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>400</v>
+        <v>625</v>
       </c>
     </row>
     <row r="133">
@@ -9806,7 +9806,7 @@
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C133" s="3" t="n">
@@ -9816,16 +9816,16 @@
         <v>5</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>16.2</v>
+        <v>3.1</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>6.5</v>
+        <v>2.3</v>
       </c>
       <c r="G133" s="3" t="n">
-        <v>461</v>
+        <v>447</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>505</v>
+        <v>400</v>
       </c>
     </row>
     <row r="134">
@@ -9880,7 +9880,7 @@
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C136" s="3" t="n">
@@ -9890,16 +9890,16 @@
         <v>5</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>5.1</v>
+        <v>85.3</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>6.2</v>
+        <v>33</v>
       </c>
       <c r="G136" s="3" t="n">
-        <v>373</v>
+        <v>1719</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>398</v>
+        <v>914</v>
       </c>
     </row>
     <row r="137">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C137" s="3" t="n">
@@ -9920,16 +9920,16 @@
         <v>5</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>18.4</v>
+        <v>5.1</v>
       </c>
       <c r="F137" s="3" t="n">
-        <v>2.5</v>
+        <v>6.2</v>
       </c>
       <c r="G137" s="3" t="n">
-        <v>1406</v>
+        <v>373</v>
       </c>
       <c r="H137" s="3" t="n">
-        <v>1450</v>
+        <v>398</v>
       </c>
     </row>
     <row r="138">
@@ -9940,7 +9940,7 @@
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C138" s="3" t="n">
@@ -9950,16 +9950,16 @@
         <v>5</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>23.3</v>
+        <v>18.4</v>
       </c>
       <c r="F138" s="3" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="G138" s="3" t="n">
-        <v>2122</v>
+        <v>1406</v>
       </c>
       <c r="H138" s="3" t="n">
-        <v>437</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="139">
@@ -9970,7 +9970,7 @@
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C139" s="3" t="n">
@@ -9980,16 +9980,16 @@
         <v>5</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>46.4</v>
+        <v>23.3</v>
       </c>
       <c r="F139" s="3" t="n">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="G139" s="3" t="n">
-        <v>2635</v>
+        <v>2122</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>910</v>
+        <v>437</v>
       </c>
     </row>
     <row r="140">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C140" s="3" t="n">
@@ -10010,16 +10010,16 @@
         <v>5</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>15.8</v>
+        <v>46.4</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>7.3</v>
+        <v>2.8</v>
       </c>
       <c r="G140" s="3" t="n">
-        <v>2104</v>
+        <v>2635</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>1168</v>
+        <v>910</v>
       </c>
     </row>
     <row r="141">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C141" s="3" t="n">
@@ -10040,16 +10040,16 @@
         <v>5</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>58.2</v>
+        <v>15.8</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>67.5</v>
+        <v>7.3</v>
       </c>
       <c r="G141" s="3" t="n">
-        <v>2020</v>
+        <v>2104</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>2502</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="142">
@@ -10060,7 +10060,7 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C142" s="3" t="n">
@@ -10070,16 +10070,16 @@
         <v>5</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>6.6</v>
+        <v>58.2</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>1.5</v>
+        <v>67.5</v>
       </c>
       <c r="G142" s="3" t="n">
-        <v>882</v>
+        <v>2020</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>410</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="143">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C143" s="3" t="n">
@@ -10100,16 +10100,16 @@
         <v>5</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>85.3</v>
+        <v>6.6</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>33</v>
+        <v>1.5</v>
       </c>
       <c r="G143" s="3" t="n">
-        <v>1719</v>
+        <v>882</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>914</v>
+        <v>410</v>
       </c>
     </row>
     <row r="144">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C146" s="3" t="n">
@@ -10174,16 +10174,16 @@
         <v>5</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>15.9</v>
+        <v>49.1</v>
       </c>
       <c r="F146" s="3" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G146" s="3" t="n">
-        <v>995</v>
+        <v>4022</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>1144</v>
+        <v>2269</v>
       </c>
     </row>
     <row r="147">
@@ -10194,7 +10194,7 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C147" s="3" t="n">
@@ -10204,16 +10204,16 @@
         <v>5</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>28.3</v>
+        <v>15.9</v>
       </c>
       <c r="F147" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>17</v>
       </c>
       <c r="G147" s="3" t="n">
-        <v>2257</v>
+        <v>995</v>
       </c>
       <c r="H147" s="3" t="n">
-        <v>2653</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="148">
@@ -10224,7 +10224,7 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C148" s="3" t="n">
@@ -10234,16 +10234,16 @@
         <v>5</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>123.2</v>
+        <v>28.3</v>
       </c>
       <c r="F148" s="3" t="n">
-        <v>11.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G148" s="3" t="n">
-        <v>12125</v>
+        <v>2257</v>
       </c>
       <c r="H148" s="3" t="n">
-        <v>1127</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="149">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C149" s="3" t="n">
@@ -10264,16 +10264,16 @@
         <v>5</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>215</v>
+        <v>123.2</v>
       </c>
       <c r="F149" s="3" t="n">
-        <v>45.4</v>
+        <v>11.4</v>
       </c>
       <c r="G149" s="3" t="n">
-        <v>12207</v>
+        <v>12125</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>3534</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="150">
@@ -10284,7 +10284,7 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C150" s="3" t="n">
@@ -10294,16 +10294,16 @@
         <v>5</v>
       </c>
       <c r="E150" s="3" t="n">
-        <v>28.5</v>
+        <v>215</v>
       </c>
       <c r="F150" s="3" t="n">
-        <v>31.3</v>
+        <v>45.4</v>
       </c>
       <c r="G150" s="3" t="n">
-        <v>3792</v>
+        <v>12207</v>
       </c>
       <c r="H150" s="3" t="n">
-        <v>4252</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="151">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C151" s="3" t="n">
@@ -10324,16 +10324,16 @@
         <v>5</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>14.9</v>
+        <v>28.5</v>
       </c>
       <c r="F151" s="3" t="n">
-        <v>91.8</v>
+        <v>31.3</v>
       </c>
       <c r="G151" s="3" t="n">
-        <v>4088</v>
+        <v>3792</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>4564</v>
+        <v>4252</v>
       </c>
     </row>
     <row r="152">
@@ -10344,7 +10344,7 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C152" s="3" t="n">
@@ -10354,16 +10354,16 @@
         <v>5</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>24.1</v>
+        <v>14.9</v>
       </c>
       <c r="F152" s="3" t="n">
-        <v>18.2</v>
+        <v>91.8</v>
       </c>
       <c r="G152" s="3" t="n">
-        <v>3090</v>
+        <v>4088</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>2325</v>
+        <v>4564</v>
       </c>
     </row>
     <row r="153">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C153" s="3" t="n">
@@ -10384,16 +10384,16 @@
         <v>5</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>49.1</v>
+        <v>24.1</v>
       </c>
       <c r="F153" s="3" t="n">
-        <v>26</v>
+        <v>18.2</v>
       </c>
       <c r="G153" s="3" t="n">
-        <v>4022</v>
+        <v>3090</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>2269</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="154">
@@ -10448,7 +10448,7 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C156" s="3" t="n">
@@ -10458,16 +10458,16 @@
         <v>13</v>
       </c>
       <c r="E156" s="3" t="n">
-        <v>20.2</v>
+        <v>55.2</v>
       </c>
       <c r="F156" s="3" t="n">
-        <v>11.5</v>
+        <v>19.4</v>
       </c>
       <c r="G156" s="3" t="n">
-        <v>2950</v>
+        <v>5382</v>
       </c>
       <c r="H156" s="3" t="n">
-        <v>2992</v>
+        <v>3684</v>
       </c>
     </row>
     <row r="157">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C157" s="3" t="n">
@@ -10488,16 +10488,16 @@
         <v>13</v>
       </c>
       <c r="E157" s="3" t="n">
-        <v>36.7</v>
+        <v>20.2</v>
       </c>
       <c r="F157" s="3" t="n">
-        <v>14.1</v>
+        <v>11.5</v>
       </c>
       <c r="G157" s="3" t="n">
-        <v>4469</v>
+        <v>2950</v>
       </c>
       <c r="H157" s="3" t="n">
-        <v>5794</v>
+        <v>2992</v>
       </c>
     </row>
     <row r="158">
@@ -10508,7 +10508,7 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C158" s="3" t="n">
@@ -10518,16 +10518,16 @@
         <v>13</v>
       </c>
       <c r="E158" s="3" t="n">
-        <v>216.9</v>
+        <v>36.7</v>
       </c>
       <c r="F158" s="3" t="n">
-        <v>19.2</v>
+        <v>14.1</v>
       </c>
       <c r="G158" s="3" t="n">
-        <v>21639</v>
+        <v>4469</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>4816</v>
+        <v>5794</v>
       </c>
     </row>
     <row r="159">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C159" s="3" t="n">
@@ -10548,16 +10548,16 @@
         <v>13</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>403.6</v>
+        <v>216.9</v>
       </c>
       <c r="F159" s="3" t="n">
-        <v>24.2</v>
+        <v>19.2</v>
       </c>
       <c r="G159" s="3" t="n">
-        <v>26420</v>
+        <v>21639</v>
       </c>
       <c r="H159" s="3" t="n">
-        <v>4274</v>
+        <v>4816</v>
       </c>
     </row>
     <row r="160">
@@ -10568,7 +10568,7 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C160" s="3" t="n">
@@ -10578,16 +10578,16 @@
         <v>13</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>23.8</v>
+        <v>403.6</v>
       </c>
       <c r="F160" s="3" t="n">
-        <v>12.4</v>
+        <v>24.2</v>
       </c>
       <c r="G160" s="3" t="n">
-        <v>5301</v>
+        <v>26420</v>
       </c>
       <c r="H160" s="3" t="n">
-        <v>4174</v>
+        <v>4274</v>
       </c>
     </row>
     <row r="161">
@@ -10598,7 +10598,7 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C161" s="3" t="n">
@@ -10608,16 +10608,16 @@
         <v>13</v>
       </c>
       <c r="E161" s="3" t="n">
-        <v>148.4</v>
+        <v>23.8</v>
       </c>
       <c r="F161" s="3" t="n">
-        <v>53.2</v>
+        <v>12.4</v>
       </c>
       <c r="G161" s="3" t="n">
-        <v>8482</v>
+        <v>5301</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>6029</v>
+        <v>4174</v>
       </c>
     </row>
     <row r="162">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C162" s="3" t="n">
@@ -10638,16 +10638,16 @@
         <v>13</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>24.9</v>
+        <v>148.4</v>
       </c>
       <c r="F162" s="3" t="n">
-        <v>10.7</v>
+        <v>53.2</v>
       </c>
       <c r="G162" s="3" t="n">
-        <v>4599</v>
+        <v>8482</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>3363</v>
+        <v>6029</v>
       </c>
     </row>
     <row r="163">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C163" s="3" t="n">
@@ -10668,16 +10668,16 @@
         <v>13</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>55.2</v>
+        <v>24.9</v>
       </c>
       <c r="F163" s="3" t="n">
-        <v>19.4</v>
+        <v>10.7</v>
       </c>
       <c r="G163" s="3" t="n">
-        <v>5382</v>
+        <v>4599</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>3684</v>
+        <v>3363</v>
       </c>
     </row>
     <row r="164">
@@ -10732,7 +10732,7 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C166" s="3" t="n">
@@ -10742,16 +10742,16 @@
         <v>15</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>112.9</v>
+        <v>127.3</v>
       </c>
       <c r="F166" s="3" t="n">
-        <v>36.2</v>
+        <v>13.9</v>
       </c>
       <c r="G166" s="3" t="n">
-        <v>6770</v>
+        <v>14964</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>3997</v>
+        <v>3852</v>
       </c>
     </row>
     <row r="167">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C167" s="3" t="n">
@@ -10772,16 +10772,16 @@
         <v>15</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>46.5</v>
+        <v>112.9</v>
       </c>
       <c r="F167" s="3" t="n">
-        <v>27.4</v>
+        <v>36.2</v>
       </c>
       <c r="G167" s="3" t="n">
-        <v>4576</v>
+        <v>6770</v>
       </c>
       <c r="H167" s="3" t="n">
-        <v>7110</v>
+        <v>3997</v>
       </c>
     </row>
     <row r="168">
@@ -10792,7 +10792,7 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C168" s="3" t="n">
@@ -10802,16 +10802,16 @@
         <v>15</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>104.4</v>
+        <v>46.5</v>
       </c>
       <c r="F168" s="3" t="n">
-        <v>8.4</v>
+        <v>27.4</v>
       </c>
       <c r="G168" s="3" t="n">
-        <v>11040</v>
+        <v>4576</v>
       </c>
       <c r="H168" s="3" t="n">
-        <v>2846</v>
+        <v>7110</v>
       </c>
     </row>
     <row r="169">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C169" s="3" t="n">
@@ -10832,16 +10832,16 @@
         <v>15</v>
       </c>
       <c r="E169" s="3" t="n">
-        <v>207.4</v>
+        <v>104.4</v>
       </c>
       <c r="F169" s="3" t="n">
-        <v>35</v>
+        <v>8.4</v>
       </c>
       <c r="G169" s="3" t="n">
-        <v>13181</v>
+        <v>11040</v>
       </c>
       <c r="H169" s="3" t="n">
-        <v>5387</v>
+        <v>2846</v>
       </c>
     </row>
     <row r="170">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C170" s="3" t="n">
@@ -10862,16 +10862,16 @@
         <v>15</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>51</v>
+        <v>207.4</v>
       </c>
       <c r="F170" s="3" t="n">
-        <v>30.9</v>
+        <v>35</v>
       </c>
       <c r="G170" s="3" t="n">
-        <v>7733</v>
+        <v>13181</v>
       </c>
       <c r="H170" s="3" t="n">
-        <v>6028</v>
+        <v>5387</v>
       </c>
     </row>
     <row r="171">
@@ -10882,7 +10882,7 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C171" s="3" t="n">
@@ -10892,16 +10892,16 @@
         <v>15</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>261.4</v>
+        <v>51</v>
       </c>
       <c r="F171" s="3" t="n">
-        <v>4.9</v>
+        <v>30.9</v>
       </c>
       <c r="G171" s="3" t="n">
-        <v>8491</v>
+        <v>7733</v>
       </c>
       <c r="H171" s="3" t="n">
-        <v>9964</v>
+        <v>6028</v>
       </c>
     </row>
     <row r="172">
@@ -10912,26 +10912,26 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C172" s="3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D172" s="3" t="n">
         <v>15</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>68.5</v>
+        <v>261.4</v>
       </c>
       <c r="F172" s="3" t="n">
-        <v>6.1</v>
+        <v>4.9</v>
       </c>
       <c r="G172" s="3" t="n">
-        <v>9102</v>
+        <v>8491</v>
       </c>
       <c r="H172" s="3" t="n">
-        <v>2272</v>
+        <v>9964</v>
       </c>
     </row>
     <row r="173">
@@ -10942,26 +10942,26 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C173" s="3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D173" s="3" t="n">
         <v>15</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>127.3</v>
+        <v>68.5</v>
       </c>
       <c r="F173" s="3" t="n">
-        <v>13.9</v>
+        <v>6.1</v>
       </c>
       <c r="G173" s="3" t="n">
-        <v>14964</v>
+        <v>9102</v>
       </c>
       <c r="H173" s="3" t="n">
-        <v>3852</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="174">
@@ -11016,7 +11016,7 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C176" s="3" t="n">
@@ -11026,16 +11026,16 @@
         <v>15</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>34.3</v>
+        <v>99.2</v>
       </c>
       <c r="F176" s="3" t="n">
-        <v>17.2</v>
+        <v>40.9</v>
       </c>
       <c r="G176" s="3" t="n">
-        <v>2605</v>
+        <v>9182</v>
       </c>
       <c r="H176" s="3" t="n">
-        <v>2457</v>
+        <v>3814</v>
       </c>
     </row>
     <row r="177">
@@ -11046,7 +11046,7 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C177" s="3" t="n">
@@ -11056,16 +11056,16 @@
         <v>15</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>35.9</v>
+        <v>34.3</v>
       </c>
       <c r="F177" s="3" t="n">
-        <v>8.1</v>
+        <v>17.2</v>
       </c>
       <c r="G177" s="3" t="n">
-        <v>2824</v>
+        <v>2605</v>
       </c>
       <c r="H177" s="3" t="n">
-        <v>3526</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="178">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C178" s="3" t="n">
@@ -11086,16 +11086,16 @@
         <v>15</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>51</v>
+        <v>35.9</v>
       </c>
       <c r="F178" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="G178" s="3" t="n">
-        <v>5025</v>
+        <v>2824</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>2956</v>
+        <v>3526</v>
       </c>
     </row>
     <row r="179">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C179" s="3" t="n">
@@ -11116,16 +11116,16 @@
         <v>15</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>118</v>
+        <v>51</v>
       </c>
       <c r="F179" s="3" t="n">
-        <v>23.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G179" s="3" t="n">
-        <v>6724</v>
+        <v>5025</v>
       </c>
       <c r="H179" s="3" t="n">
-        <v>2578</v>
+        <v>2956</v>
       </c>
     </row>
     <row r="180">
@@ -11136,7 +11136,7 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C180" s="3" t="n">
@@ -11146,16 +11146,16 @@
         <v>15</v>
       </c>
       <c r="E180" s="3" t="n">
-        <v>33.4</v>
+        <v>118</v>
       </c>
       <c r="F180" s="3" t="n">
-        <v>23.1</v>
+        <v>23.2</v>
       </c>
       <c r="G180" s="3" t="n">
-        <v>4725</v>
+        <v>6724</v>
       </c>
       <c r="H180" s="3" t="n">
-        <v>4363</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="181">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C181" s="3" t="n">
@@ -11176,16 +11176,16 @@
         <v>15</v>
       </c>
       <c r="E181" s="3" t="n">
-        <v>379.9</v>
+        <v>33.4</v>
       </c>
       <c r="F181" s="3" t="n">
-        <v>53.5</v>
+        <v>23.1</v>
       </c>
       <c r="G181" s="3" t="n">
-        <v>11856</v>
+        <v>4725</v>
       </c>
       <c r="H181" s="3" t="n">
-        <v>3124</v>
+        <v>4363</v>
       </c>
     </row>
     <row r="182">
@@ -11196,7 +11196,7 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C182" s="3" t="n">
@@ -11206,16 +11206,16 @@
         <v>15</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>28.6</v>
+        <v>379.9</v>
       </c>
       <c r="F182" s="3" t="n">
-        <v>4.7</v>
+        <v>53.5</v>
       </c>
       <c r="G182" s="3" t="n">
-        <v>3956</v>
+        <v>11856</v>
       </c>
       <c r="H182" s="3" t="n">
-        <v>1439</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="183">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C183" s="3" t="n">
@@ -11236,16 +11236,16 @@
         <v>15</v>
       </c>
       <c r="E183" s="3" t="n">
-        <v>99.2</v>
+        <v>28.6</v>
       </c>
       <c r="F183" s="3" t="n">
-        <v>40.9</v>
+        <v>4.7</v>
       </c>
       <c r="G183" s="3" t="n">
-        <v>9182</v>
+        <v>3956</v>
       </c>
       <c r="H183" s="3" t="n">
-        <v>3814</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="184">
@@ -11300,7 +11300,7 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C186" s="3" t="n">
@@ -11310,16 +11310,16 @@
         <v>17</v>
       </c>
       <c r="E186" s="3" t="n">
-        <v>177.8</v>
+        <v>223.3</v>
       </c>
       <c r="F186" s="3" t="n">
-        <v>91.3</v>
+        <v>54.1</v>
       </c>
       <c r="G186" s="3" t="n">
-        <v>11419</v>
+        <v>16462</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>7137</v>
+        <v>8449</v>
       </c>
     </row>
     <row r="187">
@@ -11330,7 +11330,7 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C187" s="3" t="n">
@@ -11340,16 +11340,16 @@
         <v>17</v>
       </c>
       <c r="E187" s="3" t="n">
-        <v>200.5</v>
+        <v>177.8</v>
       </c>
       <c r="F187" s="3" t="n">
-        <v>43.1</v>
+        <v>91.3</v>
       </c>
       <c r="G187" s="3" t="n">
-        <v>16531</v>
+        <v>11419</v>
       </c>
       <c r="H187" s="3" t="n">
-        <v>20116</v>
+        <v>7137</v>
       </c>
     </row>
     <row r="188">
@@ -11360,7 +11360,7 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C188" s="3" t="n">
@@ -11370,16 +11370,16 @@
         <v>17</v>
       </c>
       <c r="E188" s="3" t="n">
-        <v>216.2</v>
+        <v>200.5</v>
       </c>
       <c r="F188" s="3" t="n">
-        <v>20.6</v>
+        <v>43.1</v>
       </c>
       <c r="G188" s="3" t="n">
-        <v>20783</v>
+        <v>16531</v>
       </c>
       <c r="H188" s="3" t="n">
-        <v>4235</v>
+        <v>20116</v>
       </c>
     </row>
     <row r="189">
@@ -11390,7 +11390,7 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C189" s="3" t="n">
@@ -11400,16 +11400,16 @@
         <v>17</v>
       </c>
       <c r="E189" s="3" t="n">
-        <v>268</v>
+        <v>216.2</v>
       </c>
       <c r="F189" s="3" t="n">
-        <v>58.5</v>
+        <v>20.6</v>
       </c>
       <c r="G189" s="3" t="n">
-        <v>15430</v>
+        <v>20783</v>
       </c>
       <c r="H189" s="3" t="n">
-        <v>6072</v>
+        <v>4235</v>
       </c>
     </row>
     <row r="190">
@@ -11420,7 +11420,7 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C190" s="3" t="n">
@@ -11430,16 +11430,16 @@
         <v>17</v>
       </c>
       <c r="E190" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>268</v>
       </c>
       <c r="F190" s="3" t="n">
-        <v>55.4</v>
+        <v>58.5</v>
       </c>
       <c r="G190" s="3" t="n">
-        <v>13016</v>
+        <v>15430</v>
       </c>
       <c r="H190" s="3" t="n">
-        <v>10272</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="191">
@@ -11450,7 +11450,7 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C191" s="3" t="n">
@@ -11460,16 +11460,16 @@
         <v>17</v>
       </c>
       <c r="E191" s="3" t="n">
-        <v>568.7</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="F191" s="3" t="n">
-        <v>72</v>
+        <v>55.4</v>
       </c>
       <c r="G191" s="3" t="n">
-        <v>21205</v>
+        <v>13016</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>8626</v>
+        <v>10272</v>
       </c>
     </row>
     <row r="192">
@@ -11480,7 +11480,7 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C192" s="3" t="n">
@@ -11490,16 +11490,16 @@
         <v>17</v>
       </c>
       <c r="E192" s="3" t="n">
-        <v>85.90000000000001</v>
+        <v>568.7</v>
       </c>
       <c r="F192" s="3" t="n">
-        <v>5.1</v>
+        <v>72</v>
       </c>
       <c r="G192" s="3" t="n">
-        <v>12364</v>
+        <v>21205</v>
       </c>
       <c r="H192" s="3" t="n">
-        <v>2668</v>
+        <v>8626</v>
       </c>
     </row>
     <row r="193">
@@ -11510,26 +11510,26 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C193" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D193" s="3" t="n">
         <v>17</v>
       </c>
       <c r="E193" s="3" t="n">
-        <v>60.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="F193" s="3" t="n">
-        <v>94.8</v>
+        <v>5.1</v>
       </c>
       <c r="G193" s="3" t="n">
-        <v>5761</v>
+        <v>12364</v>
       </c>
       <c r="H193" s="3" t="n">
-        <v>4503</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="194">
@@ -11584,7 +11584,7 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>GPT-5.5</t>
+          <t>GLM 5.1</t>
         </is>
       </c>
       <c r="C196" s="3" t="n">
@@ -11594,16 +11594,16 @@
         <v>17</v>
       </c>
       <c r="E196" s="3" t="n">
-        <v>58.1</v>
+        <v>22.8</v>
       </c>
       <c r="F196" s="3" t="n">
-        <v>31.4</v>
+        <v>322.2</v>
       </c>
       <c r="G196" s="3" t="n">
-        <v>3813</v>
+        <v>807</v>
       </c>
       <c r="H196" s="3" t="n">
-        <v>3233</v>
+        <v>19147</v>
       </c>
     </row>
     <row r="197">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>claude-opus-4.6</t>
+          <t>GPT-5.5</t>
         </is>
       </c>
       <c r="C197" s="3" t="n">
@@ -11624,16 +11624,16 @@
         <v>17</v>
       </c>
       <c r="E197" s="3" t="n">
-        <v>194.8</v>
+        <v>58.1</v>
       </c>
       <c r="F197" s="3" t="n">
-        <v>36.9</v>
+        <v>31.4</v>
       </c>
       <c r="G197" s="3" t="n">
-        <v>16312</v>
+        <v>3813</v>
       </c>
       <c r="H197" s="3" t="n">
-        <v>19092</v>
+        <v>3233</v>
       </c>
     </row>
     <row r="198">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-lite-260428</t>
+          <t>claude-opus-4.6</t>
         </is>
       </c>
       <c r="C198" s="3" t="n">
@@ -11654,16 +11654,16 @@
         <v>17</v>
       </c>
       <c r="E198" s="3" t="n">
-        <v>178.8</v>
+        <v>194.8</v>
       </c>
       <c r="F198" s="3" t="n">
-        <v>21.2</v>
+        <v>36.9</v>
       </c>
       <c r="G198" s="3" t="n">
-        <v>16554</v>
+        <v>16312</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>5384</v>
+        <v>19092</v>
       </c>
     </row>
     <row r="199">
@@ -11674,7 +11674,7 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>doubao-seed-2-0-pro-260215</t>
+          <t>doubao-seed-2-0-lite-260428</t>
         </is>
       </c>
       <c r="C199" s="3" t="n">
@@ -11684,16 +11684,16 @@
         <v>17</v>
       </c>
       <c r="E199" s="3" t="n">
-        <v>457.7</v>
+        <v>178.8</v>
       </c>
       <c r="F199" s="3" t="n">
-        <v>6.8</v>
+        <v>21.2</v>
       </c>
       <c r="G199" s="3" t="n">
-        <v>25869</v>
+        <v>16554</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>2559</v>
+        <v>5384</v>
       </c>
     </row>
     <row r="200">
@@ -11704,7 +11704,7 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>gemini-3.1-pro-preview</t>
+          <t>doubao-seed-2-0-pro-260215</t>
         </is>
       </c>
       <c r="C200" s="3" t="n">
@@ -11714,16 +11714,16 @@
         <v>17</v>
       </c>
       <c r="E200" s="3" t="n">
-        <v>101.8</v>
+        <v>457.7</v>
       </c>
       <c r="F200" s="3" t="n">
-        <v>65.7</v>
+        <v>6.8</v>
       </c>
       <c r="G200" s="3" t="n">
-        <v>14767</v>
+        <v>25869</v>
       </c>
       <c r="H200" s="3" t="n">
-        <v>8344</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="201">
@@ -11734,7 +11734,7 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>kimi-k2.6</t>
+          <t>gemini-3.1-pro-preview</t>
         </is>
       </c>
       <c r="C201" s="3" t="n">
@@ -11744,16 +11744,16 @@
         <v>17</v>
       </c>
       <c r="E201" s="3" t="n">
-        <v>426.9</v>
+        <v>101.8</v>
       </c>
       <c r="F201" s="3" t="n">
-        <v>125.9</v>
+        <v>65.7</v>
       </c>
       <c r="G201" s="3" t="n">
-        <v>27181</v>
+        <v>14767</v>
       </c>
       <c r="H201" s="3" t="n">
-        <v>6874</v>
+        <v>8344</v>
       </c>
     </row>
     <row r="202">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>deepseek-v4-flash</t>
+          <t>kimi-k2.6</t>
         </is>
       </c>
       <c r="C202" s="3" t="n">
@@ -11774,16 +11774,16 @@
         <v>17</v>
       </c>
       <c r="E202" s="3" t="n">
-        <v>90.90000000000001</v>
+        <v>426.9</v>
       </c>
       <c r="F202" s="3" t="n">
-        <v>1.7</v>
+        <v>125.9</v>
       </c>
       <c r="G202" s="3" t="n">
-        <v>11772</v>
+        <v>27181</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>1803</v>
+        <v>6874</v>
       </c>
     </row>
     <row r="203">
@@ -11794,7 +11794,7 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>GLM 5.1</t>
+          <t>deepseek-v4-flash</t>
         </is>
       </c>
       <c r="C203" s="3" t="n">
@@ -11804,16 +11804,16 @@
         <v>17</v>
       </c>
       <c r="E203" s="3" t="n">
-        <v>22.8</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="F203" s="3" t="n">
-        <v>322.2</v>
+        <v>1.7</v>
       </c>
       <c r="G203" s="3" t="n">
-        <v>807</v>
+        <v>11772</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>19147</v>
+        <v>1803</v>
       </c>
     </row>
     <row r="204">

</xml_diff>